<commit_message>
cleaned up some code; re-ran estimates for July 10, 2024
</commit_message>
<xml_diff>
--- a/output/sfsr_inseason_ests_sy24_2024-07-09_08-58-23.xlsx
+++ b/output/sfsr_inseason_ests_sy24_2024-07-09_08-58-23.xlsx
@@ -1,99 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\sf_salmon_harvest\output\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A2E8B8D-7AD7-41BF-81C4-75284BC373A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="16440" windowHeight="28590" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="tag_exp_rel_group" sheetId="1" r:id="rId1"/>
     <sheet name="exp_summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="22">
-  <si>
-    <t>rel_group</t>
-  </si>
-  <si>
-    <t>rel_year</t>
-  </si>
-  <si>
-    <t>ocean_age</t>
-  </si>
-  <si>
-    <t>node</t>
-  </si>
-  <si>
-    <t>n_tags</t>
-  </si>
-  <si>
-    <t>n_tags_exp</t>
-  </si>
-  <si>
-    <t>KNOXB - NOR</t>
-  </si>
-  <si>
-    <t>KRS_D</t>
-  </si>
-  <si>
-    <t>SFG</t>
-  </si>
-  <si>
-    <t>LGR - HOR</t>
-  </si>
-  <si>
-    <t>KRS_U</t>
-  </si>
-  <si>
-    <t>LGR - NOR</t>
-  </si>
-  <si>
-    <t>McCall - Integrated</t>
-  </si>
-  <si>
-    <t>McCall - Segregated</t>
-  </si>
-  <si>
-    <t>SFSRKT - NOR</t>
-  </si>
-  <si>
-    <t>age</t>
-  </si>
-  <si>
-    <t>eff_est</t>
-  </si>
-  <si>
-    <t>eff_se</t>
-  </si>
-  <si>
-    <t>tot_est</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-  <si>
-    <t>Adults</t>
-  </si>
-  <si>
-    <t>Jacks</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -141,21 +64,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -193,7 +108,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -227,7 +142,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -262,10 +176,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -438,39 +351,55 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>6</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rel_group</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>rel_year</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ocean_age</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>node</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>n_tags</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>n_tags_exp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>KNOXB - NOR</t>
+        </is>
       </c>
       <c r="B2">
         <v>2021</v>
       </c>
-      <c r="D2" t="s">
-        <v>7</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E2">
         <v>1</v>
@@ -479,15 +408,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>6</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>KNOXB - NOR</t>
+        </is>
       </c>
       <c r="B3">
         <v>2021</v>
       </c>
-      <c r="D3" t="s">
-        <v>8</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E3">
         <v>1</v>
@@ -496,15 +429,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>9</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LGR - HOR</t>
+        </is>
       </c>
       <c r="B4">
         <v>2024</v>
       </c>
-      <c r="D4" t="s">
-        <v>7</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E4">
         <v>26</v>
@@ -513,15 +450,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>9</v>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LGR - HOR</t>
+        </is>
       </c>
       <c r="B5">
         <v>2024</v>
       </c>
-      <c r="D5" t="s">
-        <v>10</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E5">
         <v>27</v>
@@ -530,15 +471,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>9</v>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LGR - HOR</t>
+        </is>
       </c>
       <c r="B6">
         <v>2024</v>
       </c>
-      <c r="D6" t="s">
-        <v>8</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E6">
         <v>53</v>
@@ -547,15 +492,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>11</v>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LGR - NOR</t>
+        </is>
       </c>
       <c r="B7">
         <v>2024</v>
       </c>
-      <c r="D7" t="s">
-        <v>7</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E7">
         <v>81</v>
@@ -564,15 +513,19 @@
         <v>405</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>11</v>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LGR - NOR</t>
+        </is>
       </c>
       <c r="B8">
         <v>2024</v>
       </c>
-      <c r="D8" t="s">
-        <v>10</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E8">
         <v>86</v>
@@ -581,15 +534,19 @@
         <v>430</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>11</v>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LGR - NOR</t>
+        </is>
       </c>
       <c r="B9">
         <v>2024</v>
       </c>
-      <c r="D9" t="s">
-        <v>8</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E9">
         <v>250</v>
@@ -598,9 +555,11 @@
         <v>1250</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>12</v>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
       </c>
       <c r="B10">
         <v>2021</v>
@@ -608,8 +567,10 @@
       <c r="C10">
         <v>3</v>
       </c>
-      <c r="D10" t="s">
-        <v>7</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E10">
         <v>4</v>
@@ -618,9 +579,11 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>12</v>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
       </c>
       <c r="B11">
         <v>2021</v>
@@ -628,8 +591,10 @@
       <c r="C11">
         <v>3</v>
       </c>
-      <c r="D11" t="s">
-        <v>10</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E11">
         <v>5</v>
@@ -638,9 +603,11 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>12</v>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
       </c>
       <c r="B12">
         <v>2021</v>
@@ -648,8 +615,10 @@
       <c r="C12">
         <v>3</v>
       </c>
-      <c r="D12" t="s">
-        <v>8</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E12">
         <v>6</v>
@@ -658,9 +627,11 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>12</v>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
       </c>
       <c r="B13">
         <v>2022</v>
@@ -668,8 +639,10 @@
       <c r="C13">
         <v>2</v>
       </c>
-      <c r="D13" t="s">
-        <v>7</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E13">
         <v>31</v>
@@ -678,9 +651,11 @@
         <v>221</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>12</v>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
       </c>
       <c r="B14">
         <v>2022</v>
@@ -688,8 +663,10 @@
       <c r="C14">
         <v>2</v>
       </c>
-      <c r="D14" t="s">
-        <v>10</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E14">
         <v>35</v>
@@ -698,9 +675,11 @@
         <v>247</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>12</v>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
       </c>
       <c r="B15">
         <v>2022</v>
@@ -708,8 +687,10 @@
       <c r="C15">
         <v>2</v>
       </c>
-      <c r="D15" t="s">
-        <v>8</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E15">
         <v>33</v>
@@ -718,9 +699,11 @@
         <v>223</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>12</v>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
       </c>
       <c r="B16">
         <v>2023</v>
@@ -728,8 +711,10 @@
       <c r="C16">
         <v>1</v>
       </c>
-      <c r="D16" t="s">
-        <v>7</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E16">
         <v>12</v>
@@ -738,9 +723,11 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>12</v>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
       </c>
       <c r="B17">
         <v>2023</v>
@@ -748,8 +735,10 @@
       <c r="C17">
         <v>1</v>
       </c>
-      <c r="D17" t="s">
-        <v>10</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E17">
         <v>14</v>
@@ -758,9 +747,11 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>12</v>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
       </c>
       <c r="B18">
         <v>2023</v>
@@ -768,8 +759,10 @@
       <c r="C18">
         <v>1</v>
       </c>
-      <c r="D18" t="s">
-        <v>8</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E18">
         <v>15</v>
@@ -778,9 +771,11 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>13</v>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
       </c>
       <c r="B19">
         <v>2021</v>
@@ -788,8 +783,10 @@
       <c r="C19">
         <v>3</v>
       </c>
-      <c r="D19" t="s">
-        <v>7</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E19">
         <v>1</v>
@@ -798,9 +795,11 @@
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>13</v>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
       </c>
       <c r="B20">
         <v>2021</v>
@@ -808,8 +807,10 @@
       <c r="C20">
         <v>3</v>
       </c>
-      <c r="D20" t="s">
-        <v>10</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E20">
         <v>1</v>
@@ -818,9 +819,11 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>13</v>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
       </c>
       <c r="B21">
         <v>2021</v>
@@ -828,8 +831,10 @@
       <c r="C21">
         <v>3</v>
       </c>
-      <c r="D21" t="s">
-        <v>8</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E21">
         <v>1</v>
@@ -838,9 +843,11 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>13</v>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
       </c>
       <c r="B22">
         <v>2022</v>
@@ -848,8 +855,10 @@
       <c r="C22">
         <v>2</v>
       </c>
-      <c r="D22" t="s">
-        <v>7</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E22">
         <v>18</v>
@@ -858,9 +867,11 @@
         <v>631</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>13</v>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
       </c>
       <c r="B23">
         <v>2022</v>
@@ -868,8 +879,10 @@
       <c r="C23">
         <v>2</v>
       </c>
-      <c r="D23" t="s">
-        <v>10</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E23">
         <v>18</v>
@@ -878,9 +891,11 @@
         <v>631</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>13</v>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
       </c>
       <c r="B24">
         <v>2022</v>
@@ -888,8 +903,10 @@
       <c r="C24">
         <v>2</v>
       </c>
-      <c r="D24" t="s">
-        <v>8</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E24">
         <v>17</v>
@@ -898,9 +915,11 @@
         <v>477</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>13</v>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
       </c>
       <c r="B25">
         <v>2023</v>
@@ -908,8 +927,10 @@
       <c r="C25">
         <v>1</v>
       </c>
-      <c r="D25" t="s">
-        <v>7</v>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E25">
         <v>14</v>
@@ -918,9 +939,11 @@
         <v>453</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>13</v>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
       </c>
       <c r="B26">
         <v>2023</v>
@@ -928,8 +951,10 @@
       <c r="C26">
         <v>1</v>
       </c>
-      <c r="D26" t="s">
-        <v>10</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E26">
         <v>13</v>
@@ -938,9 +963,11 @@
         <v>452</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>13</v>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
       </c>
       <c r="B27">
         <v>2023</v>
@@ -948,8 +975,10 @@
       <c r="C27">
         <v>1</v>
       </c>
-      <c r="D27" t="s">
-        <v>8</v>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E27">
         <v>10</v>
@@ -958,15 +987,19 @@
         <v>285</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>14</v>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SFSRKT - NOR</t>
+        </is>
       </c>
       <c r="B28">
         <v>2020</v>
       </c>
-      <c r="D28" t="s">
-        <v>7</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E28">
         <v>2</v>
@@ -975,15 +1008,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>14</v>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SFSRKT - NOR</t>
+        </is>
       </c>
       <c r="B29">
         <v>2020</v>
       </c>
-      <c r="D29" t="s">
-        <v>10</v>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E29">
         <v>2</v>
@@ -992,15 +1029,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>14</v>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SFSRKT - NOR</t>
+        </is>
       </c>
       <c r="B30">
         <v>2020</v>
       </c>
-      <c r="D30" t="s">
-        <v>8</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E30">
         <v>2</v>
@@ -1009,15 +1050,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>14</v>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SFSRKT - NOR</t>
+        </is>
       </c>
       <c r="B31">
         <v>2021</v>
       </c>
-      <c r="D31" t="s">
-        <v>7</v>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E31">
         <v>5</v>
@@ -1026,15 +1071,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>14</v>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SFSRKT - NOR</t>
+        </is>
       </c>
       <c r="B32">
         <v>2021</v>
       </c>
-      <c r="D32" t="s">
-        <v>10</v>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E32">
         <v>6</v>
@@ -1043,15 +1092,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>14</v>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SFSRKT - NOR</t>
+        </is>
       </c>
       <c r="B33">
         <v>2021</v>
       </c>
-      <c r="D33" t="s">
-        <v>8</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E33">
         <v>7</v>
@@ -1060,15 +1113,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>14</v>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SFSRKT - NOR</t>
+        </is>
       </c>
       <c r="B34">
         <v>2022</v>
       </c>
-      <c r="D34" t="s">
-        <v>7</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="E34">
         <v>2</v>
@@ -1077,15 +1134,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>14</v>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SFSRKT - NOR</t>
+        </is>
       </c>
       <c r="B35">
         <v>2022</v>
       </c>
-      <c r="D35" t="s">
-        <v>10</v>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>KRS_U</t>
+        </is>
       </c>
       <c r="E35">
         <v>1</v>
@@ -1094,15 +1155,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>14</v>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SFSRKT - NOR</t>
+        </is>
       </c>
       <c r="B36">
         <v>2022</v>
       </c>
-      <c r="D36" t="s">
-        <v>8</v>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="E36">
         <v>4</v>
@@ -1117,54 +1182,67 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="17.81640625" customWidth="1"/>
-    <col min="2" max="2" width="6.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.90625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rel_group</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>node</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n_tags</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>n_tags_exp</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>eff_est</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>eff_se</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>tot_est</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LGR - NOR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="D2">
         <v>250</v>
@@ -1173,24 +1251,30 @@
         <v>1250</v>
       </c>
       <c r="F2">
-        <v>0.83364140480591498</v>
+        <v>0.833641404805915</v>
       </c>
       <c r="G2">
-        <v>9.3996535477191886E-3</v>
+        <v>0.009399653547719189</v>
       </c>
       <c r="H2">
         <v>1499</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LGR - NOR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="D3">
         <v>81</v>
@@ -1199,24 +1283,30 @@
         <v>405</v>
       </c>
       <c r="F3">
-        <v>0.87449392712550611</v>
+        <v>0.8744939271255061</v>
       </c>
       <c r="G3">
-        <v>6.7268763625038929E-3</v>
+        <v>0.006726876362503893</v>
       </c>
       <c r="H3">
         <v>463</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Adults</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="D4">
         <v>39</v>
@@ -1225,24 +1315,30 @@
         <v>259</v>
       </c>
       <c r="F4">
-        <v>0.83364140480591498</v>
+        <v>0.833641404805915</v>
       </c>
       <c r="G4">
-        <v>9.3996535477191886E-3</v>
+        <v>0.009399653547719189</v>
       </c>
       <c r="H4">
         <v>311</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Jacks</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="D5">
         <v>15</v>
@@ -1251,24 +1347,30 @@
         <v>56</v>
       </c>
       <c r="F5">
-        <v>0.83364140480591498</v>
+        <v>0.833641404805915</v>
       </c>
       <c r="G5">
-        <v>9.3996535477191886E-3</v>
+        <v>0.009399653547719189</v>
       </c>
       <c r="H5">
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>7</v>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Adults</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="D6">
         <v>35</v>
@@ -1277,24 +1379,30 @@
         <v>243</v>
       </c>
       <c r="F6">
-        <v>0.87449392712550611</v>
+        <v>0.8744939271255061</v>
       </c>
       <c r="G6">
-        <v>6.7268763625038929E-3</v>
+        <v>0.006726876362503893</v>
       </c>
       <c r="H6">
         <v>278</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" t="s">
-        <v>7</v>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>McCall - Integrated</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Jacks</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="D7">
         <v>12</v>
@@ -1303,24 +1411,30 @@
         <v>53</v>
       </c>
       <c r="F7">
-        <v>0.87449392712550611</v>
+        <v>0.8744939271255061</v>
       </c>
       <c r="G7">
-        <v>6.7268763625038929E-3</v>
+        <v>0.006726876362503893</v>
       </c>
       <c r="H7">
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Adults</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="D8">
         <v>18</v>
@@ -1329,24 +1443,30 @@
         <v>528</v>
       </c>
       <c r="F8">
-        <v>0.83364140480591498</v>
+        <v>0.833641404805915</v>
       </c>
       <c r="G8">
-        <v>9.3996535477191886E-3</v>
+        <v>0.009399653547719189</v>
       </c>
       <c r="H8">
         <v>633</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Jacks</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
       </c>
       <c r="D9">
         <v>10</v>
@@ -1355,24 +1475,30 @@
         <v>285</v>
       </c>
       <c r="F9">
-        <v>0.83364140480591498</v>
+        <v>0.833641404805915</v>
       </c>
       <c r="G9">
-        <v>9.3996535477191886E-3</v>
+        <v>0.009399653547719189</v>
       </c>
       <c r="H9">
         <v>342</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" t="s">
-        <v>7</v>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Adults</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="D10">
         <v>19</v>
@@ -1381,24 +1507,30 @@
         <v>682</v>
       </c>
       <c r="F10">
-        <v>0.87449392712550611</v>
+        <v>0.8744939271255061</v>
       </c>
       <c r="G10">
-        <v>6.7268763625038929E-3</v>
+        <v>0.006726876362503893</v>
       </c>
       <c r="H10">
         <v>780</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>7</v>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>McCall - Segregated</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Jacks</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KRS_D</t>
+        </is>
       </c>
       <c r="D11">
         <v>14</v>
@@ -1407,10 +1539,10 @@
         <v>453</v>
       </c>
       <c r="F11">
-        <v>0.87449392712550611</v>
+        <v>0.8744939271255061</v>
       </c>
       <c r="G11">
-        <v>6.7268763625038929E-3</v>
+        <v>0.006726876362503893</v>
       </c>
       <c r="H11">
         <v>518</v>

</xml_diff>